<commit_message>
Update Ordinary Kriging Zinc analysis notebook
</commit_message>
<xml_diff>
--- a/soil.xlsx
+++ b/soil.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\ASUS\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Tugas-Kelompok-ADS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5278FCDD-8B9C-414B-AB35-0B332A9AD087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9411BABA-D678-4B15-AE9A-728692FA7DB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>x</t>
   </si>
@@ -40,6 +40,9 @@
   </si>
   <si>
     <t>zinc</t>
+  </si>
+  <si>
+    <t>log_zinc</t>
   </si>
 </sst>
 </file>
@@ -570,13 +573,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C156"/>
+  <dimension ref="A1:D156"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -586,8 +589,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="1">
         <v>181072</v>
       </c>
@@ -597,8 +603,12 @@
       <c r="C2">
         <v>1022</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="D2">
+        <f>LN(C2+1)</f>
+        <v>6.9304947659516261</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="1">
         <v>181025</v>
       </c>
@@ -608,8 +618,12 @@
       <c r="C3">
         <v>1141</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="D3">
+        <f t="shared" ref="D3:D66" si="0">LN(C3+1)</f>
+        <v>7.0405363902159559</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="1">
         <v>181165</v>
       </c>
@@ -619,8 +633,12 @@
       <c r="C4">
         <v>640</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>6.4630294569206699</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="1">
         <v>181298</v>
       </c>
@@ -630,8 +648,12 @@
       <c r="C5">
         <v>257</v>
       </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>5.5529595849216173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="1">
         <v>181307</v>
       </c>
@@ -641,8 +663,12 @@
       <c r="C6">
         <v>269</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>5.598421958998375</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="1">
         <v>181390</v>
       </c>
@@ -652,8 +678,12 @@
       <c r="C7">
         <v>281</v>
       </c>
-    </row>
-    <row r="8" spans="1:3">
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>5.6419070709381138</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="1">
         <v>181165</v>
       </c>
@@ -663,8 +693,12 @@
       <c r="C8">
         <v>346</v>
       </c>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>5.8493247799468593</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" s="1">
         <v>181027</v>
       </c>
@@ -674,8 +708,12 @@
       <c r="C9">
         <v>406</v>
       </c>
-    </row>
-    <row r="10" spans="1:3">
+      <c r="D9">
+        <f t="shared" si="0"/>
+        <v>6.0088131854425946</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="1">
         <v>181060</v>
       </c>
@@ -685,8 +723,12 @@
       <c r="C10">
         <v>347</v>
       </c>
-    </row>
-    <row r="11" spans="1:3">
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>5.8522024797744745</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" s="1">
         <v>181232</v>
       </c>
@@ -696,8 +738,12 @@
       <c r="C11">
         <v>183</v>
       </c>
-    </row>
-    <row r="12" spans="1:3">
+      <c r="D11">
+        <f t="shared" si="0"/>
+        <v>5.2149357576089859</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" s="1">
         <v>181191</v>
       </c>
@@ -707,8 +753,12 @@
       <c r="C12">
         <v>189</v>
       </c>
-    </row>
-    <row r="13" spans="1:3">
+      <c r="D12">
+        <f t="shared" si="0"/>
+        <v>5.2470240721604862</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13" s="1">
         <v>181032</v>
       </c>
@@ -718,8 +768,12 @@
       <c r="C13">
         <v>251</v>
       </c>
-    </row>
-    <row r="14" spans="1:3">
+      <c r="D13">
+        <f t="shared" si="0"/>
+        <v>5.5294290875114234</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" s="1">
         <v>180874</v>
       </c>
@@ -729,8 +783,12 @@
       <c r="C14">
         <v>1096</v>
       </c>
-    </row>
-    <row r="15" spans="1:3">
+      <c r="D14">
+        <f t="shared" si="0"/>
+        <v>7.00033446027523</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15" s="1">
         <v>180969</v>
       </c>
@@ -740,8 +798,12 @@
       <c r="C15">
         <v>504</v>
       </c>
-    </row>
-    <row r="16" spans="1:3">
+      <c r="D15">
+        <f t="shared" si="0"/>
+        <v>6.2245584292753602</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16" s="1">
         <v>181011</v>
       </c>
@@ -751,8 +813,12 @@
       <c r="C16">
         <v>326</v>
       </c>
-    </row>
-    <row r="17" spans="1:3">
+      <c r="D16">
+        <f t="shared" si="0"/>
+        <v>5.7899601708972535</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
       <c r="A17" s="1">
         <v>180830</v>
       </c>
@@ -762,8 +828,12 @@
       <c r="C17">
         <v>1032</v>
       </c>
-    </row>
-    <row r="18" spans="1:3">
+      <c r="D17">
+        <f t="shared" si="0"/>
+        <v>6.9402224691196386</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18" s="1">
         <v>180763</v>
       </c>
@@ -773,8 +843,12 @@
       <c r="C18">
         <v>606</v>
       </c>
-    </row>
-    <row r="19" spans="1:3">
+      <c r="D18">
+        <f t="shared" si="0"/>
+        <v>6.4085287910594984</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
       <c r="A19" s="1">
         <v>180694</v>
       </c>
@@ -784,8 +858,12 @@
       <c r="C19">
         <v>711</v>
       </c>
-    </row>
-    <row r="20" spans="1:3">
+      <c r="D19">
+        <f t="shared" si="0"/>
+        <v>6.5680779114119758</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
       <c r="A20" s="1">
         <v>180625</v>
       </c>
@@ -795,8 +873,12 @@
       <c r="C20">
         <v>735</v>
       </c>
-    </row>
-    <row r="21" spans="1:3">
+      <c r="D20">
+        <f t="shared" si="0"/>
+        <v>6.6012301187288767</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21" s="1">
         <v>180555</v>
       </c>
@@ -806,8 +888,12 @@
       <c r="C21">
         <v>1052</v>
       </c>
-    </row>
-    <row r="22" spans="1:3">
+      <c r="D21">
+        <f t="shared" si="0"/>
+        <v>6.9593985121339754</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22" s="1">
         <v>180642</v>
       </c>
@@ -817,8 +903,12 @@
       <c r="C22">
         <v>673</v>
       </c>
-    </row>
-    <row r="23" spans="1:3">
+      <c r="D22">
+        <f t="shared" si="0"/>
+        <v>6.513230110912307</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
       <c r="A23" s="1">
         <v>180704</v>
       </c>
@@ -828,8 +918,12 @@
       <c r="C23">
         <v>402</v>
       </c>
-    </row>
-    <row r="24" spans="1:3">
+      <c r="D23">
+        <f t="shared" si="0"/>
+        <v>5.9989365619466826</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
       <c r="A24" s="1">
         <v>180704</v>
       </c>
@@ -839,8 +933,12 @@
       <c r="C24">
         <v>343</v>
       </c>
-    </row>
-    <row r="25" spans="1:3">
+      <c r="D24">
+        <f t="shared" si="0"/>
+        <v>5.8406416573733981</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
       <c r="A25" s="1">
         <v>181153</v>
       </c>
@@ -850,8 +948,12 @@
       <c r="C25">
         <v>218</v>
       </c>
-    </row>
-    <row r="26" spans="1:3">
+      <c r="D25">
+        <f t="shared" si="0"/>
+        <v>5.389071729816501</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
       <c r="A26" s="1">
         <v>181147</v>
       </c>
@@ -861,8 +963,12 @@
       <c r="C26">
         <v>200</v>
       </c>
-    </row>
-    <row r="27" spans="1:3">
+      <c r="D26">
+        <f t="shared" si="0"/>
+        <v>5.3033049080590757</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
       <c r="A27" s="1">
         <v>181167</v>
       </c>
@@ -872,8 +978,12 @@
       <c r="C27">
         <v>194</v>
       </c>
-    </row>
-    <row r="28" spans="1:3">
+      <c r="D27">
+        <f t="shared" si="0"/>
+        <v>5.2729995585637468</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
       <c r="A28" s="1">
         <v>181008</v>
       </c>
@@ -883,8 +993,12 @@
       <c r="C28">
         <v>207</v>
       </c>
-    </row>
-    <row r="29" spans="1:3">
+      <c r="D28">
+        <f t="shared" si="0"/>
+        <v>5.3375380797013179</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
       <c r="A29" s="1">
         <v>180973</v>
       </c>
@@ -894,8 +1008,12 @@
       <c r="C29">
         <v>180</v>
       </c>
-    </row>
-    <row r="30" spans="1:3">
+      <c r="D29">
+        <f t="shared" si="0"/>
+        <v>5.1984970312658261</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
       <c r="A30" s="1">
         <v>180916</v>
       </c>
@@ -905,8 +1023,12 @@
       <c r="C30">
         <v>240</v>
       </c>
-    </row>
-    <row r="31" spans="1:3">
+      <c r="D30">
+        <f t="shared" si="0"/>
+        <v>5.4847969334906548</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
       <c r="A31" s="1">
         <v>181352</v>
       </c>
@@ -916,8 +1038,12 @@
       <c r="C31">
         <v>180</v>
       </c>
-    </row>
-    <row r="32" spans="1:3">
+      <c r="D31">
+        <f t="shared" si="0"/>
+        <v>5.1984970312658261</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
       <c r="A32" s="1">
         <v>181133</v>
       </c>
@@ -927,8 +1053,12 @@
       <c r="C32">
         <v>208</v>
       </c>
-    </row>
-    <row r="33" spans="1:3">
+      <c r="D32">
+        <f t="shared" si="0"/>
+        <v>5.3423342519648109</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
       <c r="A33" s="1">
         <v>180878</v>
       </c>
@@ -938,8 +1068,12 @@
       <c r="C33">
         <v>198</v>
       </c>
-    </row>
-    <row r="34" spans="1:3">
+      <c r="D33">
+        <f t="shared" si="0"/>
+        <v>5.2933048247244923</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
       <c r="A34" s="1">
         <v>180829</v>
       </c>
@@ -949,8 +1083,12 @@
       <c r="C34">
         <v>250</v>
       </c>
-    </row>
-    <row r="35" spans="1:3">
+      <c r="D34">
+        <f t="shared" si="0"/>
+        <v>5.5254529391317835</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
       <c r="A35" s="1">
         <v>180954</v>
       </c>
@@ -960,8 +1098,12 @@
       <c r="C35">
         <v>192</v>
       </c>
-    </row>
-    <row r="36" spans="1:3">
+      <c r="D35">
+        <f t="shared" si="0"/>
+        <v>5.2626901889048856</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
       <c r="A36" s="1">
         <v>180956</v>
       </c>
@@ -971,8 +1113,12 @@
       <c r="C36">
         <v>213</v>
       </c>
-    </row>
-    <row r="37" spans="1:3">
+      <c r="D36">
+        <f t="shared" si="0"/>
+        <v>5.3659760150218512</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
       <c r="A37" s="1">
         <v>180710</v>
       </c>
@@ -982,8 +1128,12 @@
       <c r="C37">
         <v>321</v>
       </c>
-    </row>
-    <row r="38" spans="1:3">
+      <c r="D37">
+        <f t="shared" si="0"/>
+        <v>5.7745515455444085</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
       <c r="A38" s="1">
         <v>180632</v>
       </c>
@@ -993,8 +1143,12 @@
       <c r="C38">
         <v>569</v>
       </c>
-    </row>
-    <row r="39" spans="1:3">
+      <c r="D38">
+        <f t="shared" si="0"/>
+        <v>6.3456363608285962</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
       <c r="A39" s="1">
         <v>180530</v>
       </c>
@@ -1004,8 +1158,12 @@
       <c r="C39">
         <v>833</v>
       </c>
-    </row>
-    <row r="40" spans="1:3">
+      <c r="D39">
+        <f t="shared" si="0"/>
+        <v>6.7262334023587469</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
       <c r="A40" s="1">
         <v>180478</v>
       </c>
@@ -1015,8 +1173,12 @@
       <c r="C40">
         <v>906</v>
       </c>
-    </row>
-    <row r="41" spans="1:3">
+      <c r="D40">
+        <f t="shared" si="0"/>
+        <v>6.8101424501151362</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
       <c r="A41" s="1">
         <v>180383</v>
       </c>
@@ -1026,8 +1188,12 @@
       <c r="C41">
         <v>1454</v>
       </c>
-    </row>
-    <row r="42" spans="1:3">
+      <c r="D41">
+        <f t="shared" si="0"/>
+        <v>7.2827611796055933</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
       <c r="A42" s="1">
         <v>180494</v>
       </c>
@@ -1037,8 +1203,12 @@
       <c r="C42">
         <v>298</v>
       </c>
-    </row>
-    <row r="43" spans="1:3">
+      <c r="D42">
+        <f t="shared" si="0"/>
+        <v>5.7004435733906869</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
       <c r="A43" s="1">
         <v>180561</v>
       </c>
@@ -1048,8 +1218,12 @@
       <c r="C43">
         <v>167</v>
       </c>
-    </row>
-    <row r="44" spans="1:3">
+      <c r="D43">
+        <f t="shared" si="0"/>
+        <v>5.1239639794032588</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
       <c r="A44" s="1">
         <v>180451</v>
       </c>
@@ -1059,8 +1233,12 @@
       <c r="C44">
         <v>176</v>
       </c>
-    </row>
-    <row r="45" spans="1:3">
+      <c r="D44">
+        <f t="shared" si="0"/>
+        <v>5.1761497325738288</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
       <c r="A45" s="1">
         <v>180410</v>
       </c>
@@ -1070,8 +1248,12 @@
       <c r="C45">
         <v>258</v>
       </c>
-    </row>
-    <row r="46" spans="1:3">
+      <c r="D45">
+        <f t="shared" si="0"/>
+        <v>5.5568280616995374</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
       <c r="A46" s="1">
         <v>180355</v>
       </c>
@@ -1081,8 +1263,12 @@
       <c r="C46">
         <v>746</v>
       </c>
-    </row>
-    <row r="47" spans="1:3">
+      <c r="D46">
+        <f t="shared" si="0"/>
+        <v>6.6160651851328174</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
       <c r="A47" s="1">
         <v>180292</v>
       </c>
@@ -1092,8 +1278,12 @@
       <c r="C47">
         <v>746</v>
       </c>
-    </row>
-    <row r="48" spans="1:3">
+      <c r="D47">
+        <f t="shared" si="0"/>
+        <v>6.6160651851328174</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
       <c r="A48" s="1">
         <v>180283</v>
       </c>
@@ -1103,8 +1293,12 @@
       <c r="C48">
         <v>464</v>
       </c>
-    </row>
-    <row r="49" spans="1:3">
+      <c r="D48">
+        <f t="shared" si="0"/>
+        <v>6.1420374055873559</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
       <c r="A49" s="1">
         <v>180282</v>
       </c>
@@ -1114,8 +1308,12 @@
       <c r="C49">
         <v>365</v>
       </c>
-    </row>
-    <row r="50" spans="1:3">
+      <c r="D49">
+        <f t="shared" si="0"/>
+        <v>5.9026333334013659</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
       <c r="A50" s="1">
         <v>180270</v>
       </c>
@@ -1125,8 +1323,12 @@
       <c r="C50">
         <v>282</v>
       </c>
-    </row>
-    <row r="51" spans="1:3">
+      <c r="D50">
+        <f t="shared" si="0"/>
+        <v>5.6454468976432377</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
       <c r="A51" s="1">
         <v>180199</v>
       </c>
@@ -1136,8 +1338,12 @@
       <c r="C51">
         <v>375</v>
       </c>
-    </row>
-    <row r="52" spans="1:3">
+      <c r="D51">
+        <f t="shared" si="0"/>
+        <v>5.9295891433898946</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
       <c r="A52" s="1">
         <v>180135</v>
       </c>
@@ -1147,8 +1353,12 @@
       <c r="C52">
         <v>222</v>
       </c>
-    </row>
-    <row r="53" spans="1:3">
+      <c r="D52">
+        <f t="shared" si="0"/>
+        <v>5.4071717714601188</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
       <c r="A53" s="1">
         <v>180237</v>
       </c>
@@ -1158,8 +1368,12 @@
       <c r="C53">
         <v>812</v>
       </c>
-    </row>
-    <row r="54" spans="1:3">
+      <c r="D53">
+        <f t="shared" si="0"/>
+        <v>6.7007311095478101</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
       <c r="A54" s="1">
         <v>180103</v>
       </c>
@@ -1169,8 +1383,12 @@
       <c r="C54">
         <v>1548</v>
       </c>
-    </row>
-    <row r="55" spans="1:3">
+      <c r="D54">
+        <f t="shared" si="0"/>
+        <v>7.3453648404168685</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
       <c r="A55" s="1">
         <v>179973</v>
       </c>
@@ -1180,8 +1398,12 @@
       <c r="C55">
         <v>1839</v>
       </c>
-    </row>
-    <row r="56" spans="1:3">
+      <c r="D55">
+        <f t="shared" si="0"/>
+        <v>7.5175208506030309</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
       <c r="A56" s="1">
         <v>179826</v>
       </c>
@@ -1191,8 +1413,12 @@
       <c r="C56">
         <v>1528</v>
       </c>
-    </row>
-    <row r="57" spans="1:3">
+      <c r="D56">
+        <f t="shared" si="0"/>
+        <v>7.3323692059290622</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
       <c r="A57" s="1">
         <v>179687</v>
       </c>
@@ -1202,8 +1428,12 @@
       <c r="C57">
         <v>933</v>
       </c>
-    </row>
-    <row r="58" spans="1:3">
+      <c r="D57">
+        <f t="shared" si="0"/>
+        <v>6.8394764382288429</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
       <c r="A58" s="1">
         <v>179792</v>
       </c>
@@ -1213,8 +1443,12 @@
       <c r="C58">
         <v>432</v>
       </c>
-    </row>
-    <row r="59" spans="1:3">
+      <c r="D58">
+        <f t="shared" si="0"/>
+        <v>6.0707377280024897</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
       <c r="A59" s="1">
         <v>179902</v>
       </c>
@@ -1224,8 +1458,12 @@
       <c r="C59">
         <v>550</v>
       </c>
-    </row>
-    <row r="60" spans="1:3">
+      <c r="D59">
+        <f t="shared" si="0"/>
+        <v>6.3117348091529148</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
       <c r="A60" s="1">
         <v>180100</v>
       </c>
@@ -1235,8 +1473,12 @@
       <c r="C60">
         <v>1571</v>
       </c>
-    </row>
-    <row r="61" spans="1:3">
+      <c r="D60">
+        <f t="shared" si="0"/>
+        <v>7.360103972989152</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
       <c r="A61" s="1">
         <v>179604</v>
       </c>
@@ -1246,8 +1488,12 @@
       <c r="C61">
         <v>1190</v>
       </c>
-    </row>
-    <row r="62" spans="1:3">
+      <c r="D61">
+        <f t="shared" si="0"/>
+        <v>7.0825485693552999</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
       <c r="A62" s="1">
         <v>179526</v>
       </c>
@@ -1257,8 +1503,12 @@
       <c r="C62">
         <v>907</v>
       </c>
-    </row>
-    <row r="63" spans="1:3">
+      <c r="D62">
+        <f t="shared" si="0"/>
+        <v>6.8112443786012937</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
       <c r="A63" s="1">
         <v>179495</v>
       </c>
@@ -1268,8 +1518,12 @@
       <c r="C63">
         <v>761</v>
       </c>
-    </row>
-    <row r="64" spans="1:3">
+      <c r="D63">
+        <f t="shared" si="0"/>
+        <v>6.6359465556866466</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
       <c r="A64" s="1">
         <v>179489</v>
       </c>
@@ -1279,8 +1533,12 @@
       <c r="C64">
         <v>659</v>
       </c>
-    </row>
-    <row r="65" spans="1:3">
+      <c r="D64">
+        <f t="shared" si="0"/>
+        <v>6.4922398350204711</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
       <c r="A65" s="1">
         <v>179414</v>
       </c>
@@ -1290,8 +1548,12 @@
       <c r="C65">
         <v>643</v>
       </c>
-    </row>
-    <row r="66" spans="1:3">
+      <c r="D65">
+        <f t="shared" si="0"/>
+        <v>6.4676987261043539</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
       <c r="A66" s="1">
         <v>179334</v>
       </c>
@@ -1301,8 +1563,12 @@
       <c r="C66">
         <v>801</v>
       </c>
-    </row>
-    <row r="67" spans="1:3">
+      <c r="D66">
+        <f t="shared" si="0"/>
+        <v>6.6871086078665147</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
       <c r="A67" s="1">
         <v>179255</v>
       </c>
@@ -1312,8 +1578,12 @@
       <c r="C67">
         <v>784</v>
       </c>
-    </row>
-    <row r="68" spans="1:3">
+      <c r="D67">
+        <f t="shared" ref="D67:D130" si="1">LN(C67+1)</f>
+        <v>6.6656837177824082</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
       <c r="A68" s="1">
         <v>179470</v>
       </c>
@@ -1323,8 +1593,12 @@
       <c r="C68">
         <v>1060</v>
       </c>
-    </row>
-    <row r="69" spans="1:3">
+      <c r="D68">
+        <f t="shared" si="1"/>
+        <v>6.9669671386139829</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
       <c r="A69" s="1">
         <v>179692</v>
       </c>
@@ -1334,8 +1608,12 @@
       <c r="C69">
         <v>119</v>
       </c>
-    </row>
-    <row r="70" spans="1:3">
+      <c r="D69">
+        <f t="shared" si="1"/>
+        <v>4.7874917427820458</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
       <c r="A70" s="1">
         <v>179852</v>
       </c>
@@ -1345,8 +1623,12 @@
       <c r="C70">
         <v>778</v>
       </c>
-    </row>
-    <row r="71" spans="1:3">
+      <c r="D70">
+        <f t="shared" si="1"/>
+        <v>6.6580110458707482</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
       <c r="A71" s="1">
         <v>179140</v>
       </c>
@@ -1356,8 +1638,12 @@
       <c r="C71">
         <v>703</v>
       </c>
-    </row>
-    <row r="72" spans="1:3">
+      <c r="D71">
+        <f t="shared" si="1"/>
+        <v>6.5567783561580422</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
       <c r="A72" s="1">
         <v>179128</v>
       </c>
@@ -1367,8 +1653,12 @@
       <c r="C72">
         <v>676</v>
       </c>
-    </row>
-    <row r="73" spans="1:3">
+      <c r="D72">
+        <f t="shared" si="1"/>
+        <v>6.517671272912275</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
       <c r="A73" s="1">
         <v>179065</v>
       </c>
@@ -1378,8 +1668,12 @@
       <c r="C73">
         <v>793</v>
       </c>
-    </row>
-    <row r="74" spans="1:3">
+      <c r="D73">
+        <f t="shared" si="1"/>
+        <v>6.6770834612471361</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
       <c r="A74" s="1">
         <v>179007</v>
       </c>
@@ -1389,8 +1683,12 @@
       <c r="C74">
         <v>685</v>
       </c>
-    </row>
-    <row r="75" spans="1:3">
+      <c r="D74">
+        <f t="shared" si="1"/>
+        <v>6.5308776277258849</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4">
       <c r="A75" s="1">
         <v>179110</v>
       </c>
@@ -1400,8 +1698,12 @@
       <c r="C75">
         <v>593</v>
       </c>
-    </row>
-    <row r="76" spans="1:3">
+      <c r="D75">
+        <f t="shared" si="1"/>
+        <v>6.3868793193626452</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4">
       <c r="A76" s="1">
         <v>179032</v>
       </c>
@@ -1411,8 +1713,12 @@
       <c r="C76">
         <v>549</v>
       </c>
-    </row>
-    <row r="77" spans="1:3">
+      <c r="D76">
+        <f t="shared" si="1"/>
+        <v>6.3099182782265162</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
       <c r="A77" s="1">
         <v>179095</v>
       </c>
@@ -1422,8 +1728,12 @@
       <c r="C77">
         <v>680</v>
       </c>
-    </row>
-    <row r="78" spans="1:3">
+      <c r="D77">
+        <f t="shared" si="1"/>
+        <v>6.523562306149512</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
       <c r="A78" s="1">
         <v>179058</v>
       </c>
@@ -1433,8 +1743,12 @@
       <c r="C78">
         <v>539</v>
       </c>
-    </row>
-    <row r="79" spans="1:3">
+      <c r="D78">
+        <f t="shared" si="1"/>
+        <v>6.2915691395583204</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4">
       <c r="A79" s="1">
         <v>178810</v>
       </c>
@@ -1444,8 +1758,12 @@
       <c r="C79">
         <v>560</v>
       </c>
-    </row>
-    <row r="80" spans="1:3">
+      <c r="D79">
+        <f t="shared" si="1"/>
+        <v>6.329720905522696</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4">
       <c r="A80" s="1">
         <v>178912</v>
       </c>
@@ -1455,8 +1773,12 @@
       <c r="C80">
         <v>1136</v>
       </c>
-    </row>
-    <row r="81" spans="1:3">
+      <c r="D80">
+        <f t="shared" si="1"/>
+        <v>7.0361484937505363</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4">
       <c r="A81" s="1">
         <v>178981</v>
       </c>
@@ -1466,8 +1788,12 @@
       <c r="C81">
         <v>1383</v>
       </c>
-    </row>
-    <row r="82" spans="1:3">
+      <c r="D81">
+        <f t="shared" si="1"/>
+        <v>7.2327331361776146</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4">
       <c r="A82" s="1">
         <v>179076</v>
       </c>
@@ -1477,8 +1803,12 @@
       <c r="C82">
         <v>1161</v>
       </c>
-    </row>
-    <row r="83" spans="1:3">
+      <c r="D82">
+        <f t="shared" si="1"/>
+        <v>7.0578979374118562</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4">
       <c r="A83" s="1">
         <v>180151</v>
       </c>
@@ -1488,8 +1818,12 @@
       <c r="C83">
         <v>1672</v>
       </c>
-    </row>
-    <row r="84" spans="1:3">
+      <c r="D83">
+        <f t="shared" si="1"/>
+        <v>7.4223737009868236</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4">
       <c r="A84" s="1">
         <v>179211</v>
       </c>
@@ -1499,8 +1833,12 @@
       <c r="C84">
         <v>765</v>
       </c>
-    </row>
-    <row r="85" spans="1:3">
+      <c r="D84">
+        <f t="shared" si="1"/>
+        <v>6.6411821697405911</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4">
       <c r="A85" s="1">
         <v>181118</v>
       </c>
@@ -1510,8 +1848,12 @@
       <c r="C85">
         <v>279</v>
       </c>
-    </row>
-    <row r="86" spans="1:3">
+      <c r="D85">
+        <f t="shared" si="1"/>
+        <v>5.6347896031692493</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4">
       <c r="A86" s="1">
         <v>179474</v>
       </c>
@@ -1521,8 +1863,12 @@
       <c r="C86">
         <v>241</v>
       </c>
-    </row>
-    <row r="87" spans="1:3">
+      <c r="D86">
+        <f t="shared" si="1"/>
+        <v>5.4889377261566867</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4">
       <c r="A87" s="1">
         <v>179559</v>
       </c>
@@ -1532,8 +1878,12 @@
       <c r="C87">
         <v>317</v>
       </c>
-    </row>
-    <row r="88" spans="1:3">
+      <c r="D87">
+        <f t="shared" si="1"/>
+        <v>5.7620513827801769</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
       <c r="A88" s="1">
         <v>179022</v>
       </c>
@@ -1543,8 +1893,12 @@
       <c r="C88">
         <v>545</v>
       </c>
-    </row>
-    <row r="89" spans="1:3">
+      <c r="D88">
+        <f t="shared" si="1"/>
+        <v>6.3026189757449051</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4">
       <c r="A89" s="1">
         <v>178953</v>
       </c>
@@ -1554,8 +1908,12 @@
       <c r="C89">
         <v>505</v>
       </c>
-    </row>
-    <row r="90" spans="1:3">
+      <c r="D89">
+        <f t="shared" si="1"/>
+        <v>6.2265366692874657</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4">
       <c r="A90" s="1">
         <v>178875</v>
       </c>
@@ -1565,8 +1923,12 @@
       <c r="C90">
         <v>420</v>
       </c>
-    </row>
-    <row r="91" spans="1:3">
+      <c r="D90">
+        <f t="shared" si="1"/>
+        <v>6.0426328336823811</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4">
       <c r="A91" s="1">
         <v>178803</v>
       </c>
@@ -1576,8 +1938,12 @@
       <c r="C91">
         <v>332</v>
       </c>
-    </row>
-    <row r="92" spans="1:3">
+      <c r="D91">
+        <f t="shared" si="1"/>
+        <v>5.8081424899804439</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4">
       <c r="A92" s="1">
         <v>179029</v>
       </c>
@@ -1587,8 +1953,12 @@
       <c r="C92">
         <v>400</v>
       </c>
-    </row>
-    <row r="93" spans="1:3">
+      <c r="D92">
+        <f t="shared" si="1"/>
+        <v>5.9939614273065693</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
       <c r="A93" s="1">
         <v>178605</v>
       </c>
@@ -1598,8 +1968,12 @@
       <c r="C93">
         <v>553</v>
       </c>
-    </row>
-    <row r="94" spans="1:3">
+      <c r="D93">
+        <f t="shared" si="1"/>
+        <v>6.3171646867472839</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4">
       <c r="A94" s="1">
         <v>178701</v>
       </c>
@@ -1609,8 +1983,12 @@
       <c r="C94">
         <v>577</v>
       </c>
-    </row>
-    <row r="95" spans="1:3">
+      <c r="D94">
+        <f t="shared" si="1"/>
+        <v>6.3595738686723777</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4">
       <c r="A95" s="1">
         <v>179547</v>
       </c>
@@ -1620,8 +1998,12 @@
       <c r="C95">
         <v>155</v>
       </c>
-    </row>
-    <row r="96" spans="1:3">
+      <c r="D95">
+        <f t="shared" si="1"/>
+        <v>5.0498560072495371</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4">
       <c r="A96" s="1">
         <v>179301</v>
       </c>
@@ -1631,8 +2013,12 @@
       <c r="C96">
         <v>224</v>
       </c>
-    </row>
-    <row r="97" spans="1:3">
+      <c r="D96">
+        <f t="shared" si="1"/>
+        <v>5.4161004022044201</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4">
       <c r="A97" s="1">
         <v>179405</v>
       </c>
@@ -1642,8 +2028,12 @@
       <c r="C97">
         <v>180</v>
       </c>
-    </row>
-    <row r="98" spans="1:3">
+      <c r="D97">
+        <f t="shared" si="1"/>
+        <v>5.1984970312658261</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4">
       <c r="A98" s="1">
         <v>179462</v>
       </c>
@@ -1653,8 +2043,12 @@
       <c r="C98">
         <v>226</v>
       </c>
-    </row>
-    <row r="99" spans="1:3">
+      <c r="D98">
+        <f t="shared" si="1"/>
+        <v>5.4249500174814029</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4">
       <c r="A99" s="1">
         <v>179293</v>
       </c>
@@ -1664,8 +2058,12 @@
       <c r="C99">
         <v>186</v>
       </c>
-    </row>
-    <row r="100" spans="1:3">
+      <c r="D99">
+        <f t="shared" si="1"/>
+        <v>5.2311086168545868</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4">
       <c r="A100" s="1">
         <v>179180</v>
       </c>
@@ -1675,8 +2073,12 @@
       <c r="C100">
         <v>198</v>
       </c>
-    </row>
-    <row r="101" spans="1:3">
+      <c r="D100">
+        <f t="shared" si="1"/>
+        <v>5.2933048247244923</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4">
       <c r="A101" s="1">
         <v>179206</v>
       </c>
@@ -1686,8 +2088,12 @@
       <c r="C101">
         <v>187</v>
       </c>
-    </row>
-    <row r="102" spans="1:3">
+      <c r="D101">
+        <f t="shared" si="1"/>
+        <v>5.2364419628299492</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4">
       <c r="A102" s="1">
         <v>179618</v>
       </c>
@@ -1697,8 +2103,12 @@
       <c r="C102">
         <v>199</v>
       </c>
-    </row>
-    <row r="103" spans="1:3">
+      <c r="D102">
+        <f t="shared" si="1"/>
+        <v>5.2983173665480363</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4">
       <c r="A103" s="1">
         <v>179782</v>
       </c>
@@ -1708,8 +2118,12 @@
       <c r="C103">
         <v>157</v>
       </c>
-    </row>
-    <row r="104" spans="1:3">
+      <c r="D103">
+        <f t="shared" si="1"/>
+        <v>5.0625950330269669</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4">
       <c r="A104" s="1">
         <v>179980</v>
       </c>
@@ -1719,8 +2133,12 @@
       <c r="C104">
         <v>203</v>
       </c>
-    </row>
-    <row r="105" spans="1:3">
+      <c r="D104">
+        <f t="shared" si="1"/>
+        <v>5.3181199938442161</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4">
       <c r="A105" s="1">
         <v>180067</v>
       </c>
@@ -1730,8 +2148,12 @@
       <c r="C105">
         <v>143</v>
       </c>
-    </row>
-    <row r="106" spans="1:3">
+      <c r="D105">
+        <f t="shared" si="1"/>
+        <v>4.9698132995760007</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4">
       <c r="A106" s="1">
         <v>180162</v>
       </c>
@@ -1741,8 +2163,12 @@
       <c r="C106">
         <v>136</v>
       </c>
-    </row>
-    <row r="107" spans="1:3">
+      <c r="D106">
+        <f t="shared" si="1"/>
+        <v>4.9199809258281251</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4">
       <c r="A107" s="1">
         <v>180451</v>
       </c>
@@ -1752,8 +2178,12 @@
       <c r="C107">
         <v>117</v>
       </c>
-    </row>
-    <row r="108" spans="1:3">
+      <c r="D107">
+        <f t="shared" si="1"/>
+        <v>4.7706846244656651</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4">
       <c r="A108" s="1">
         <v>180328</v>
       </c>
@@ -1763,8 +2193,12 @@
       <c r="C108">
         <v>113</v>
       </c>
-    </row>
-    <row r="109" spans="1:3">
+      <c r="D108">
+        <f t="shared" si="1"/>
+        <v>4.7361984483944957</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4">
       <c r="A109" s="1">
         <v>180276</v>
       </c>
@@ -1774,8 +2208,12 @@
       <c r="C109">
         <v>130</v>
       </c>
-    </row>
-    <row r="110" spans="1:3">
+      <c r="D109">
+        <f t="shared" si="1"/>
+        <v>4.8751973232011512</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4">
       <c r="A110" s="1">
         <v>180114</v>
       </c>
@@ -1785,8 +2223,12 @@
       <c r="C110">
         <v>192</v>
       </c>
-    </row>
-    <row r="111" spans="1:3">
+      <c r="D110">
+        <f t="shared" si="1"/>
+        <v>5.2626901889048856</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4">
       <c r="A111" s="1">
         <v>179881</v>
       </c>
@@ -1796,8 +2238,12 @@
       <c r="C111">
         <v>240</v>
       </c>
-    </row>
-    <row r="112" spans="1:3">
+      <c r="D111">
+        <f t="shared" si="1"/>
+        <v>5.4847969334906548</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4">
       <c r="A112" s="1">
         <v>179774</v>
       </c>
@@ -1807,8 +2253,12 @@
       <c r="C112">
         <v>221</v>
       </c>
-    </row>
-    <row r="113" spans="1:3">
+      <c r="D112">
+        <f t="shared" si="1"/>
+        <v>5.4026773818722793</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4">
       <c r="A113" s="1">
         <v>179657</v>
       </c>
@@ -1818,8 +2268,12 @@
       <c r="C113">
         <v>140</v>
       </c>
-    </row>
-    <row r="114" spans="1:3">
+      <c r="D113">
+        <f t="shared" si="1"/>
+        <v>4.9487598903781684</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4">
       <c r="A114" s="1">
         <v>179731</v>
       </c>
@@ -1829,8 +2283,12 @@
       <c r="C114">
         <v>128</v>
       </c>
-    </row>
-    <row r="115" spans="1:3">
+      <c r="D114">
+        <f t="shared" si="1"/>
+        <v>4.8598124043616719</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4">
       <c r="A115" s="1">
         <v>179717</v>
       </c>
@@ -1840,8 +2298,12 @@
       <c r="C115">
         <v>166</v>
       </c>
-    </row>
-    <row r="116" spans="1:3">
+      <c r="D115">
+        <f t="shared" si="1"/>
+        <v>5.1179938124167554</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4">
       <c r="A116" s="1">
         <v>179446</v>
       </c>
@@ -1851,8 +2313,12 @@
       <c r="C116">
         <v>191</v>
       </c>
-    </row>
-    <row r="117" spans="1:3">
+      <c r="D116">
+        <f t="shared" si="1"/>
+        <v>5.2574953720277815</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4">
       <c r="A117" s="1">
         <v>179524</v>
       </c>
@@ -1862,8 +2328,12 @@
       <c r="C117">
         <v>232</v>
       </c>
-    </row>
-    <row r="118" spans="1:3">
+      <c r="D117">
+        <f t="shared" si="1"/>
+        <v>5.4510384535657002</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4">
       <c r="A118" s="1">
         <v>179644</v>
       </c>
@@ -1873,8 +2343,12 @@
       <c r="C118">
         <v>203</v>
       </c>
-    </row>
-    <row r="119" spans="1:3">
+      <c r="D118">
+        <f t="shared" si="1"/>
+        <v>5.3181199938442161</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4">
       <c r="A119" s="1">
         <v>180321</v>
       </c>
@@ -1884,8 +2358,12 @@
       <c r="C119">
         <v>722</v>
       </c>
-    </row>
-    <row r="120" spans="1:3">
+      <c r="D119">
+        <f t="shared" si="1"/>
+        <v>6.5834092221587648</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4">
       <c r="A120" s="1">
         <v>180162</v>
       </c>
@@ -1895,8 +2373,12 @@
       <c r="C120">
         <v>210</v>
       </c>
-    </row>
-    <row r="121" spans="1:3">
+      <c r="D120">
+        <f t="shared" si="1"/>
+        <v>5.3518581334760666</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4">
       <c r="A121" s="1">
         <v>180029</v>
       </c>
@@ -1906,8 +2388,12 @@
       <c r="C121">
         <v>198</v>
       </c>
-    </row>
-    <row r="122" spans="1:3">
+      <c r="D121">
+        <f t="shared" si="1"/>
+        <v>5.2933048247244923</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4">
       <c r="A122" s="1">
         <v>179797</v>
       </c>
@@ -1917,8 +2403,12 @@
       <c r="C122">
         <v>139</v>
       </c>
-    </row>
-    <row r="123" spans="1:3">
+      <c r="D122">
+        <f t="shared" si="1"/>
+        <v>4.9416424226093039</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4">
       <c r="A123" s="1">
         <v>179642</v>
       </c>
@@ -1928,8 +2418,12 @@
       <c r="C123">
         <v>253</v>
       </c>
-    </row>
-    <row r="124" spans="1:3">
+      <c r="D123">
+        <f t="shared" si="1"/>
+        <v>5.5373342670185366</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4">
       <c r="A124" s="1">
         <v>179849</v>
       </c>
@@ -1939,8 +2433,12 @@
       <c r="C124">
         <v>703</v>
       </c>
-    </row>
-    <row r="125" spans="1:3">
+      <c r="D124">
+        <f t="shared" si="1"/>
+        <v>6.5567783561580422</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4">
       <c r="A125" s="1">
         <v>180265</v>
       </c>
@@ -1950,8 +2448,12 @@
       <c r="C125">
         <v>832</v>
       </c>
-    </row>
-    <row r="126" spans="1:3">
+      <c r="D125">
+        <f t="shared" si="1"/>
+        <v>6.7250336421668431</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4">
       <c r="A126" s="1">
         <v>180107</v>
       </c>
@@ -1961,8 +2463,12 @@
       <c r="C126">
         <v>262</v>
       </c>
-    </row>
-    <row r="127" spans="1:3">
+      <c r="D126">
+        <f t="shared" si="1"/>
+        <v>5.5721540321777647</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4">
       <c r="A127" s="1">
         <v>180462</v>
       </c>
@@ -1972,8 +2478,12 @@
       <c r="C127">
         <v>142</v>
       </c>
-    </row>
-    <row r="128" spans="1:3">
+      <c r="D127">
+        <f t="shared" si="1"/>
+        <v>4.962844630259907</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4">
       <c r="A128" s="1">
         <v>180478</v>
       </c>
@@ -1983,8 +2493,12 @@
       <c r="C128">
         <v>119</v>
       </c>
-    </row>
-    <row r="129" spans="1:3">
+      <c r="D128">
+        <f t="shared" si="1"/>
+        <v>4.7874917427820458</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4">
       <c r="A129" s="1">
         <v>180347</v>
       </c>
@@ -1994,8 +2508,12 @@
       <c r="C129">
         <v>152</v>
       </c>
-    </row>
-    <row r="130" spans="1:3">
+      <c r="D129">
+        <f t="shared" si="1"/>
+        <v>5.0304379213924353</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4">
       <c r="A130" s="1">
         <v>180862</v>
       </c>
@@ -2005,8 +2523,12 @@
       <c r="C130">
         <v>415</v>
       </c>
-    </row>
-    <row r="131" spans="1:3">
+      <c r="D130">
+        <f t="shared" si="1"/>
+        <v>6.0306852602612633</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4">
       <c r="A131" s="1">
         <v>180700</v>
       </c>
@@ -2016,8 +2538,12 @@
       <c r="C131">
         <v>474</v>
       </c>
-    </row>
-    <row r="132" spans="1:3">
+      <c r="D131">
+        <f t="shared" ref="D131:D156" si="2">LN(C131+1)</f>
+        <v>6.1633148040346413</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4">
       <c r="A132" s="1">
         <v>180201</v>
       </c>
@@ -2027,8 +2553,12 @@
       <c r="C132">
         <v>126</v>
       </c>
-    </row>
-    <row r="133" spans="1:3">
+      <c r="D132">
+        <f t="shared" si="2"/>
+        <v>4.8441870864585912</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4">
       <c r="A133" s="1">
         <v>180173</v>
       </c>
@@ -2038,8 +2568,12 @@
       <c r="C133">
         <v>210</v>
       </c>
-    </row>
-    <row r="134" spans="1:3">
+      <c r="D133">
+        <f t="shared" si="2"/>
+        <v>5.3518581334760666</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4">
       <c r="A134" s="1">
         <v>180923</v>
       </c>
@@ -2049,8 +2583,12 @@
       <c r="C134">
         <v>220</v>
       </c>
-    </row>
-    <row r="135" spans="1:3">
+      <c r="D134">
+        <f t="shared" si="2"/>
+        <v>5.3981627015177525</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4">
       <c r="A135" s="1">
         <v>180467</v>
       </c>
@@ -2060,8 +2598,12 @@
       <c r="C135">
         <v>133</v>
       </c>
-    </row>
-    <row r="136" spans="1:3">
+      <c r="D135">
+        <f t="shared" si="2"/>
+        <v>4.8978397999509111</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4">
       <c r="A136" s="1">
         <v>179917</v>
       </c>
@@ -2071,8 +2613,12 @@
       <c r="C136">
         <v>141</v>
       </c>
-    </row>
-    <row r="137" spans="1:3">
+      <c r="D136">
+        <f t="shared" si="2"/>
+        <v>4.9558270576012609</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4">
       <c r="A137" s="1">
         <v>179822</v>
       </c>
@@ -2082,8 +2628,12 @@
       <c r="C137">
         <v>158</v>
       </c>
-    </row>
-    <row r="138" spans="1:3">
+      <c r="D137">
+        <f t="shared" si="2"/>
+        <v>5.0689042022202315</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4">
       <c r="A138" s="1">
         <v>179991</v>
       </c>
@@ -2093,8 +2643,12 @@
       <c r="C138">
         <v>129</v>
       </c>
-    </row>
-    <row r="139" spans="1:3">
+      <c r="D138">
+        <f t="shared" si="2"/>
+        <v>4.8675344504555822</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4">
       <c r="A139" s="1">
         <v>179120</v>
       </c>
@@ -2104,8 +2658,12 @@
       <c r="C139">
         <v>206</v>
       </c>
-    </row>
-    <row r="140" spans="1:3">
+      <c r="D139">
+        <f t="shared" si="2"/>
+        <v>5.3327187932653688</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4">
       <c r="A140" s="1">
         <v>179034</v>
       </c>
@@ -2115,8 +2673,12 @@
       <c r="C140">
         <v>451</v>
       </c>
-    </row>
-    <row r="141" spans="1:3">
+      <c r="D140">
+        <f t="shared" si="2"/>
+        <v>6.1136821798322316</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4">
       <c r="A141" s="1">
         <v>179085</v>
       </c>
@@ -2126,8 +2688,12 @@
       <c r="C141">
         <v>296</v>
       </c>
-    </row>
-    <row r="142" spans="1:3">
+      <c r="D141">
+        <f t="shared" si="2"/>
+        <v>5.6937321388026998</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4">
       <c r="A142" s="1">
         <v>179236</v>
       </c>
@@ -2137,8 +2703,12 @@
       <c r="C142">
         <v>189</v>
       </c>
-    </row>
-    <row r="143" spans="1:3">
+      <c r="D142">
+        <f t="shared" si="2"/>
+        <v>5.2470240721604862</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4">
       <c r="A143" s="1">
         <v>179456</v>
       </c>
@@ -2148,8 +2718,12 @@
       <c r="C143">
         <v>154</v>
       </c>
-    </row>
-    <row r="144" spans="1:3">
+      <c r="D143">
+        <f t="shared" si="2"/>
+        <v>5.0434251169192468</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4">
       <c r="A144" s="1">
         <v>179550</v>
       </c>
@@ -2159,8 +2733,12 @@
       <c r="C144">
         <v>169</v>
       </c>
-    </row>
-    <row r="145" spans="1:3">
+      <c r="D144">
+        <f t="shared" si="2"/>
+        <v>5.1357984370502621</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4">
       <c r="A145" s="1">
         <v>179445</v>
       </c>
@@ -2170,8 +2748,12 @@
       <c r="C145">
         <v>403</v>
       </c>
-    </row>
-    <row r="146" spans="1:3">
+      <c r="D145">
+        <f t="shared" si="2"/>
+        <v>6.0014148779611505</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4">
       <c r="A146" s="1">
         <v>179337</v>
       </c>
@@ -2181,8 +2763,12 @@
       <c r="C146">
         <v>471</v>
       </c>
-    </row>
-    <row r="147" spans="1:3">
+      <c r="D146">
+        <f t="shared" si="2"/>
+        <v>6.156978985585555</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4">
       <c r="A147" s="1">
         <v>179245</v>
       </c>
@@ -2192,8 +2778,12 @@
       <c r="C147">
         <v>612</v>
       </c>
-    </row>
-    <row r="148" spans="1:3">
+      <c r="D147">
+        <f t="shared" si="2"/>
+        <v>6.4183649359362116</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4">
       <c r="A148" s="1">
         <v>179024</v>
       </c>
@@ -2203,8 +2793,12 @@
       <c r="C148">
         <v>601</v>
       </c>
-    </row>
-    <row r="149" spans="1:3">
+      <c r="D148">
+        <f t="shared" si="2"/>
+        <v>6.4002574453088208</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4">
       <c r="A149" s="1">
         <v>178786</v>
       </c>
@@ -2214,8 +2808,12 @@
       <c r="C149">
         <v>783</v>
       </c>
-    </row>
-    <row r="150" spans="1:3">
+      <c r="D149">
+        <f t="shared" si="2"/>
+        <v>6.6644090203504076</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4">
       <c r="A150" s="1">
         <v>179135</v>
       </c>
@@ -2225,8 +2823,12 @@
       <c r="C150">
         <v>258</v>
       </c>
-    </row>
-    <row r="151" spans="1:3">
+      <c r="D150">
+        <f t="shared" si="2"/>
+        <v>5.5568280616995374</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4">
       <c r="A151" s="1">
         <v>179030</v>
       </c>
@@ -2236,8 +2838,12 @@
       <c r="C151">
         <v>214</v>
       </c>
-    </row>
-    <row r="152" spans="1:3">
+      <c r="D151">
+        <f t="shared" si="2"/>
+        <v>5.3706380281276624</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4">
       <c r="A152" s="1">
         <v>179184</v>
       </c>
@@ -2247,8 +2853,12 @@
       <c r="C152">
         <v>166</v>
       </c>
-    </row>
-    <row r="153" spans="1:3">
+      <c r="D152">
+        <f t="shared" si="2"/>
+        <v>5.1179938124167554</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4">
       <c r="A153" s="1">
         <v>179085</v>
       </c>
@@ -2258,8 +2868,12 @@
       <c r="C153">
         <v>496</v>
       </c>
-    </row>
-    <row r="154" spans="1:3">
+      <c r="D153">
+        <f t="shared" si="2"/>
+        <v>6.2085900260966289</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4">
       <c r="A154" s="1">
         <v>178875</v>
       </c>
@@ -2269,8 +2883,12 @@
       <c r="C154">
         <v>342</v>
       </c>
-    </row>
-    <row r="155" spans="1:3">
+      <c r="D154">
+        <f t="shared" si="2"/>
+        <v>5.8377304471659395</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4">
       <c r="A155" s="1">
         <v>179466</v>
       </c>
@@ -2280,8 +2898,12 @@
       <c r="C155">
         <v>162</v>
       </c>
-    </row>
-    <row r="156" spans="1:3">
+      <c r="D155">
+        <f t="shared" si="2"/>
+        <v>5.0937502008067623</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4">
       <c r="A156" s="1">
         <v>180627</v>
       </c>
@@ -2290,6 +2912,10 @@
       </c>
       <c r="C156">
         <v>375</v>
+      </c>
+      <c r="D156">
+        <f t="shared" si="2"/>
+        <v>5.9295891433898946</v>
       </c>
     </row>
   </sheetData>

</xml_diff>